<commit_message>
Traitement automatique : Argis (retenter_erreurs/continuer)
</commit_message>
<xml_diff>
--- a/state/01017_argis.xlsx
+++ b/state/01017_argis.xlsx
@@ -12405,72 +12405,72 @@
       </c>
       <c r="ID3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR3" t="inlineStr">
@@ -14887,72 +14887,72 @@
       </c>
       <c r="ID4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ4" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR4" t="inlineStr">
@@ -17369,72 +17369,72 @@
       </c>
       <c r="ID5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ5" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR5" t="inlineStr">
@@ -19851,72 +19851,72 @@
       </c>
       <c r="ID6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ6" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR6" t="inlineStr">
@@ -22333,72 +22333,72 @@
       </c>
       <c r="ID7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ7" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR7" t="inlineStr">
@@ -27297,72 +27297,72 @@
       </c>
       <c r="ID9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ9" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR9" t="inlineStr">
@@ -29779,72 +29779,72 @@
       </c>
       <c r="ID10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR10" t="inlineStr">
@@ -32261,72 +32261,72 @@
       </c>
       <c r="ID11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR11" t="inlineStr">
@@ -34743,72 +34743,72 @@
       </c>
       <c r="ID12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR12" t="inlineStr">
@@ -37225,72 +37225,72 @@
       </c>
       <c r="ID13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR13" t="inlineStr">
@@ -39707,72 +39707,72 @@
       </c>
       <c r="ID14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR14" t="inlineStr">
@@ -42189,72 +42189,72 @@
       </c>
       <c r="ID15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR15" t="inlineStr">
@@ -44671,72 +44671,72 @@
       </c>
       <c r="ID16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR16" t="inlineStr">
@@ -47153,72 +47153,72 @@
       </c>
       <c r="ID17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR17" t="inlineStr">
@@ -49635,72 +49635,72 @@
       </c>
       <c r="ID18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR18" t="inlineStr">
@@ -52117,72 +52117,72 @@
       </c>
       <c r="ID19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR19" t="inlineStr">
@@ -54599,72 +54599,72 @@
       </c>
       <c r="ID20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ20" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR20" t="inlineStr">
@@ -57081,72 +57081,72 @@
       </c>
       <c r="ID21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ21" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR21" t="inlineStr">
@@ -62045,72 +62045,72 @@
       </c>
       <c r="ID23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ23" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR23" t="inlineStr">
@@ -64527,72 +64527,72 @@
       </c>
       <c r="ID24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ24" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR24" t="inlineStr">
@@ -67009,72 +67009,72 @@
       </c>
       <c r="ID25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ25" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR25" t="inlineStr">
@@ -69491,72 +69491,72 @@
       </c>
       <c r="ID26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ26" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR26" t="inlineStr">
@@ -71973,72 +71973,72 @@
       </c>
       <c r="ID27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ27" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR27" t="inlineStr">
@@ -74455,72 +74455,72 @@
       </c>
       <c r="ID28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ28" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR28" t="inlineStr">
@@ -76937,72 +76937,72 @@
       </c>
       <c r="ID29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ29" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR29" t="inlineStr">
@@ -79419,72 +79419,72 @@
       </c>
       <c r="ID30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ30" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR30" t="inlineStr">
@@ -81901,72 +81901,72 @@
       </c>
       <c r="ID31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ31" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR31" t="inlineStr">
@@ -84383,72 +84383,72 @@
       </c>
       <c r="ID32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ32" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR32" t="inlineStr">
@@ -86865,72 +86865,72 @@
       </c>
       <c r="ID33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ33" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR33" t="inlineStr">
@@ -89347,72 +89347,72 @@
       </c>
       <c r="ID34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ34" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR34" t="inlineStr">
@@ -91829,72 +91829,72 @@
       </c>
       <c r="ID35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ35" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR35" t="inlineStr">
@@ -94331,17 +94331,17 @@
       </c>
       <c r="IH36" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II36" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ36" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK36" t="inlineStr">
@@ -94366,7 +94366,7 @@
       </c>
       <c r="IO36" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP36" t="inlineStr">
@@ -96793,72 +96793,72 @@
       </c>
       <c r="ID37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ37" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR37" t="inlineStr">
@@ -99275,72 +99275,72 @@
       </c>
       <c r="ID38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ38" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR38" t="inlineStr">
@@ -101757,72 +101757,72 @@
       </c>
       <c r="ID39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ39" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR39" t="inlineStr">

</xml_diff>